<commit_message>
Actualización automática de base de datos y registro de noticias
</commit_message>
<xml_diff>
--- a/noticias_registro.xlsx
+++ b/noticias_registro.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,6 +526,94 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nathalie Cook: “Debemos crear equilibrio entre el uso de la tecnología y la defensa de nuestra ancestralidad” - adn.celam.org</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Nathalie Cook: “Debemos crear equilibrio entre el uso de la tecnología y la defensa de nuestra ancestralidad”  adn.celam.org</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4wFBVV95cUxNdUZaWmUzUTdTVFRlN0NMaUtOQy03NGpZS1RWemV1Q1QtNURxZUJNd0JNMER5OWg0eDhndFFZbTBNcm94ZGxRTnpaTkZVN21CSkMyQ1pzMDRyZ2l1UHFGUkRXT0h2WVZzZnRpYUdNMGdrNlRBSTBmcENyTWN5YzI3WUhHSF9hM0NBb2ZWWUh5VERROGRVajNmTU5uUW5yaGQ1ZVBVVnJBMDcwN2I1YzVaRkpXMjBTWXRLZVgzc2dfcUdKd3pHQVdqVlRpWmJIODFWa1ZhWkl5eW5NcHFJTVJ3WmQzSQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tecnología permite reforzar la seguridad y respuesta en el Quindío - Crónica del Quindio</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tecnología permite reforzar la seguridad y respuesta en el Quindío  Crónica del Quindio</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxQdjFqUE1nM0xhNFNiT240NlZLVHNrT3lKY3BKbEtKZlRsSjJtQXRsWVBPelMwT0VPTzI3WlZLZVJVR051SVViUFBiQzljZ2RLZWREeERZZDhNckY2WklnR0FGRzBZNXo5RVJtT3otNWk2bEpGb2QxdHlKb0E0NDJ3X2VseGJLS2k0M0haOXhiZTFRcUJrVDBkN0taYS1MV1BYQmZ6RlQ2WXY?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>¡Triunfo de Atlético Nacional en la Serie Colombia! - ESPN Argentina</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>¡Triunfo de Atlético Nacional en la Serie Colombia!  ESPN Argentina</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOM0RvU2FDRnNvaks3YlJwUXZWT28yaTdHeDRlaXlROThIdDJfZGNHeU4xREZxWHF0WlhoakVaajNsMmVVQ3NBLWE0LWkxRWpvZXlFUVFDMEVoOWpJYkpiTThXR011alFPUjR0eF9ZdDBqNVJXLWsxR3oydXBPZmVjS2pFVEgtT1ZGejFLRWMxUjhCMklqaDNONU5RNENHYVE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>La Selección Colombia Femenina Sub-20 visita el Estadio Miejski LKS Łódź - Federación Colombiana de Futbol</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>La Selección Colombia Femenina Sub-20 visita el Estadio Miejski LKS Łódź  Federación Colombiana de Futbol</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPZUtFUVUwQmxydXNRQzJ0RU5xZURZcC13RGNYVVZNbVI1OXlmdGJ3OEpVX280RGFfV2NpU3pHd3BEXzFjMFRDbVAtS0VXbkhtNlV4TlNCTzZvTGNUbktRVUlKZkJzVk1XclBnYnM3Tk8xVnZaaVRIbkpMREZwamZmdUNvNklaX25LQnkxN0FDZ05Rd0dUZ3hSMklXYzdKaWEtNU5iNkNR?oc=5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>